<commit_message>
docs(hardware): BOM MVP v0 verificado en LCSC + costos de corrida (issue #4)
</commit_message>
<xml_diff>
--- a/Hardware/BOM/bom-mvp-v0.xlsx
+++ b/Hardware/BOM/bom-mvp-v0.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="184" uniqueCount="149">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="189" uniqueCount="154">
   <si>
     <t xml:space="preserve">Bill of Materials (BOM) — MVP v0</t>
   </si>
@@ -448,22 +448,37 @@
     <t xml:space="preserve">CORREGIDO: el C72043 del issue está descontinuado (stock=1). Reemplazo verificado.</t>
   </si>
   <si>
-    <t xml:space="preserve">RESUMEN DE COSTO (USD por placa)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Subtotal componentes LCSC (config default U4b, excl. módulo U1)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Módulo LSM110A (U1) — precio GREATECH, confirmar con distribuidor</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TOTAL estimado por placa (config directa 3V)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Si se puebla el LDO regulado U4a en vez del 0Ω: sumar +$0.49 (@100u) / +$0.43 (@1ku)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Setup fees JLCPCB SMT: ~4 partes Extended ensamblables (U2, U3, BAT1, C_TX) × ~$3 = ~$12 one-time. U1 y U4a van hand-load (sin assembly).</t>
+    <t xml:space="preserve">RESUMEN DE COSTO (USD)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">@precio 100u</t>
+  </si>
+  <si>
+    <t xml:space="preserve">@precio 1ku</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Componentes LCSC por placa (config default U4b, excl. módulo U1)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Módulo LSM110A (U1) por placa — precio GREATECH, confirmar con distribuidor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">COSTO POR PLACA (1 unidad terminada, config directa 3V)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TOTAL CORRIDA 100 placas  (= costo por placa @100u × 100)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TOTAL CORRIDA 1000 placas (= costo por placa @1ku × 1000)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nota: @100u y @1ku son PRECIO UNITARIO al comprar en ese volumen (descuento). 'Por placa' ya multiplica por Qty. 'Corrida' = por placa × Nº de placas.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Si se puebla el LDO regulado U4a en vez del 0Ω: sumar +$0.49 (@100u) / +$0.43 (@1ku) por placa.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Setup fees JLCPCB SMT (one-time, no por placa): ~4 partes Extended ensamblables (U2, U3, BAT1, C_TX) × ~$3 = ~$12. U1 y U4a van hand-load (sin assembly).</t>
   </si>
   <si>
     <t xml:space="preserve">Módulo LSM110A (GREATECH): 500u=€3675 y 1000u=€7350 → €7.35/u (≈$7.94). Domina el costo; confirmar MOQ con SeongJi/GREATECH antes de presupuestar en firme.</t>
@@ -473,12 +488,13 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="\$#,##0.0000;&quot;($&quot;#,##0.0000\);\-"/>
     <numFmt numFmtId="166" formatCode="\$#,##0.00;&quot;($&quot;#,##0.00\);\-"/>
+    <numFmt numFmtId="167" formatCode="\$#,##0.00"/>
   </numFmts>
-  <fonts count="14">
+  <fonts count="15">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -562,6 +578,14 @@
       <charset val="1"/>
     </font>
     <font>
+      <b val="true"/>
+      <sz val="9"/>
+      <color rgb="FF1F3864"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
       <sz val="10"/>
       <name val="Arial"/>
       <family val="0"/>
@@ -575,7 +599,7 @@
       <charset val="1"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -597,13 +621,19 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFE2EFDA"/>
-        <bgColor rgb="FFFCE4D6"/>
+        <bgColor rgb="FFDDEBF7"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFF2CC"/>
         <bgColor rgb="FFFCE4D6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFDDEBF7"/>
+        <bgColor rgb="FFE2EFDA"/>
       </patternFill>
     </fill>
   </fills>
@@ -656,7 +686,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="23">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -717,7 +747,11 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -729,7 +763,19 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="13" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="166" fontId="14" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="14" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="6" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -763,7 +809,7 @@
       <rgbColor rgb="FF9999FF"/>
       <rgbColor rgb="FF993366"/>
       <rgbColor rgb="FFFFF2CC"/>
-      <rgbColor rgb="FFCCFFFF"/>
+      <rgbColor rgb="FFDDEBF7"/>
       <rgbColor rgb="FF660066"/>
       <rgbColor rgb="FFFF8080"/>
       <rgbColor rgb="FF0563C1"/>
@@ -985,7 +1031,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:Q27"/>
+  <dimension ref="A1:Q31"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="14"/>
@@ -1797,59 +1843,90 @@
       <c r="A21" s="14" t="s">
         <v>142</v>
       </c>
+      <c r="J21" s="15" t="s">
+        <v>143</v>
+      </c>
+      <c r="K21" s="15" t="s">
+        <v>144</v>
+      </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="15" t="s">
-        <v>143</v>
-      </c>
-      <c r="J22" s="16" t="n">
+      <c r="A22" s="16" t="s">
+        <v>145</v>
+      </c>
+      <c r="J22" s="17" t="n">
         <f aca="false">SUM(P8:P19)</f>
         <v>2.0171</v>
       </c>
-      <c r="K22" s="16" t="n">
+      <c r="K22" s="17" t="n">
         <f aca="false">SUM(Q8:Q19)</f>
         <v>1.7232</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="15" t="s">
-        <v>144</v>
-      </c>
-      <c r="J23" s="16" t="n">
+      <c r="A23" s="16" t="s">
+        <v>146</v>
+      </c>
+      <c r="J23" s="17" t="n">
         <f aca="false">P7</f>
         <v>10.1</v>
       </c>
-      <c r="K23" s="16" t="n">
+      <c r="K23" s="17" t="n">
         <f aca="false">Q7</f>
         <v>7.94</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="17" t="s">
-        <v>145</v>
-      </c>
-      <c r="J24" s="18" t="n">
+      <c r="A24" s="18" t="s">
+        <v>147</v>
+      </c>
+      <c r="J24" s="19" t="n">
         <f aca="false">J22+J23</f>
         <v>12.1171</v>
       </c>
-      <c r="K24" s="18" t="n">
+      <c r="K24" s="19" t="n">
         <f aca="false">K22+K23</f>
         <v>9.6632</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="3" t="s">
-        <v>146</v>
-      </c>
+      <c r="A25" s="20" t="s">
+        <v>148</v>
+      </c>
+      <c r="J25" s="21" t="n">
+        <f aca="false">J24*100</f>
+        <v>1211.71</v>
+      </c>
+      <c r="K25" s="22"/>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="3" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="3" t="s">
-        <v>148</v>
+      <c r="A26" s="20" t="s">
+        <v>149</v>
+      </c>
+      <c r="J26" s="22"/>
+      <c r="K26" s="21" t="n">
+        <f aca="false">K24*1000</f>
+        <v>9663.2</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="3" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="3" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="3" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="3" t="s">
+        <v>153</v>
       </c>
     </row>
   </sheetData>

</xml_diff>